<commit_message>
Initial project check in
</commit_message>
<xml_diff>
--- a/ProvarProject/templates/TestData.xlsx
+++ b/ProvarProject/templates/TestData.xlsx
@@ -1,139 +1,114 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23127"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\16156\git\provardx\ProvarProject\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zac.taylor/git/POC-Google/GooglePOC/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD9F04A-8A37-4C66-B5BF-C899B5F01B33}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC3D33A-8417-724A-B119-637B201D621B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="4050" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-29460" yWindow="2820" windowWidth="28040" windowHeight="17440" xr2:uid="{7581156E-45D0-5844-9C4C-1E315867C4A1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Property" sheetId="1" r:id="rId1"/>
-    <sheet name="Broker" sheetId="2" r:id="rId2"/>
+    <sheet name="Fill" sheetId="1" r:id="rId1"/>
+    <sheet name="TotalPUF" sheetId="2" r:id="rId2"/>
+    <sheet name="SSR" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
-  <si>
-    <t>Name</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="17">
+  <si>
+    <t>GSKU</t>
+  </si>
+  <si>
+    <t>Stores</t>
+  </si>
+  <si>
+    <t>Pegs</t>
+  </si>
+  <si>
+    <t>CardsPerPeg</t>
+  </si>
+  <si>
+    <t>Activity</t>
   </si>
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>Address</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>Beds</t>
-  </si>
-  <si>
-    <t>Baths</t>
-  </si>
-  <si>
-    <t>AskingPrice</t>
-  </si>
-  <si>
-    <t>State</t>
-  </si>
-  <si>
-    <t>Zip</t>
-  </si>
-  <si>
-    <t>Broker</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>DateContracted</t>
-  </si>
-  <si>
-    <t>DatePreMarket</t>
-  </si>
-  <si>
-    <t>DateListed</t>
-  </si>
-  <si>
-    <t>DateAgreement</t>
-  </si>
-  <si>
-    <t>ProvarDX Homebase</t>
-  </si>
-  <si>
-    <t>7112 Crossroads Blvd.</t>
-  </si>
-  <si>
-    <t>Brentwood</t>
-  </si>
-  <si>
-    <t>TN</t>
-  </si>
-  <si>
-    <t>Devy McDevin</t>
-  </si>
-  <si>
-    <t>Lead Broker</t>
-  </si>
-  <si>
-    <t>The best property in DX history!</t>
-  </si>
-  <si>
-    <t>DateClosed</t>
-  </si>
-  <si>
-    <t>555-555-5555</t>
-  </si>
-  <si>
-    <t>devy.mcdevin@provartesting.com</t>
-  </si>
-  <si>
-    <t>Available</t>
+    <t>AT20003 - 15_1000327_1-step</t>
+  </si>
+  <si>
+    <t>Regression Testing</t>
+  </si>
+  <si>
+    <t>Planned</t>
+  </si>
+  <si>
+    <t>WorkspaceId</t>
+  </si>
+  <si>
+    <t>a160m000001SqvIAAS</t>
+  </si>
+  <si>
+    <t>Retailer Launch</t>
+  </si>
+  <si>
+    <t>PrimaryReason</t>
+  </si>
+  <si>
+    <t>Override</t>
+  </si>
+  <si>
+    <t>Reason</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Units</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0;[Red]#,##0"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
+      <color theme="1"/>
+      <name val="Helvetica Neue"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -153,17 +128,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -196,7 +170,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -208,7 +182,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -255,6 +229,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -290,6 +281,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -441,25 +449,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BDEFB38-E26E-1E45-B120-D629B99624B6}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.9296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.73046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.06640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.46484375" customWidth="1"/>
-    <col min="10" max="10" width="12.73046875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.9296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.9296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.53125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.6640625" customWidth="1"/>
-    <col min="16" max="16" width="14.19921875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.5" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="19.5" customWidth="1"/>
+    <col min="7" max="7" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -479,128 +479,140 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
+      <c r="D2">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="F2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="G2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
         <v>11</v>
-      </c>
-      <c r="L1" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" t="s">
-        <v>14</v>
-      </c>
-      <c r="N1" t="s">
-        <v>15</v>
-      </c>
-      <c r="O1" t="s">
-        <v>16</v>
-      </c>
-      <c r="P1" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>300000</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2">
-        <v>37027</v>
-      </c>
-      <c r="J2" t="s">
-        <v>22</v>
-      </c>
-      <c r="K2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L2" t="s">
-        <v>24</v>
-      </c>
-      <c r="O2" s="1">
-        <v>43831</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1FBD8B1-0ABF-4BCD-89A2-C65053DDF8EA}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4876B18B-3655-F443-8FC0-35F4BD5CC0E6}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.9296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.1640625" customWidth="1"/>
+    <col min="2" max="2" width="31.5" customWidth="1"/>
+    <col min="3" max="3" width="17.5" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="D1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>27</v>
+      <c r="F2" s="3">
+        <v>50009</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{3FE0F942-8337-4DAF-ADAD-79D118B5E425}"/>
-  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{816A0B5E-7679-AE41-9C89-C0B5D45A1D99}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="31" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>2.25</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
checking in Zac's changes
</commit_message>
<xml_diff>
--- a/ProvarProject/templates/TestData.xlsx
+++ b/ProvarProject/templates/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zac.taylor/git/POC-Google/GooglePOC/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC3D33A-8417-724A-B119-637B201D621B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27599374-EBC4-3A44-AB06-17B57020C812}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29460" yWindow="2820" windowWidth="28040" windowHeight="17440" xr2:uid="{7581156E-45D0-5844-9C4C-1E315867C4A1}"/>
+    <workbookView xWindow="-26320" yWindow="2540" windowWidth="24580" windowHeight="17440" activeTab="1" xr2:uid="{7581156E-45D0-5844-9C4C-1E315867C4A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Fill" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="15">
   <si>
     <t>GSKU</t>
   </si>
@@ -50,9 +50,6 @@
     <t>CardsPerPeg</t>
   </si>
   <si>
-    <t>Activity</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -81,9 +78,6 @@
   </si>
   <si>
     <t>Reason</t>
-  </si>
-  <si>
-    <t>Notes</t>
   </si>
   <si>
     <t>Units</t>
@@ -450,16 +444,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BDEFB38-E26E-1E45-B120-D629B99624B6}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.5" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="19.5" customWidth="1"/>
-    <col min="7" max="7" width="20.33203125" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -476,18 +469,15 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>9</v>
-      </c>
-      <c r="H1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>6</v>
       </c>
       <c r="B2">
         <v>10</v>
@@ -501,14 +491,11 @@
       <c r="E2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="1" t="s">
+      <c r="F2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
         <v>10</v>
-      </c>
-      <c r="H2" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -519,54 +506,40 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4876B18B-3655-F443-8FC0-35F4BD5CC0E6}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.1640625" customWidth="1"/>
     <col min="2" max="2" width="31.5" customWidth="1"/>
-    <col min="3" max="3" width="17.5" customWidth="1"/>
-    <col min="4" max="4" width="18.33203125" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" style="2"/>
+    <col min="3" max="3" width="14.6640625" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="3">
+      <c r="D2" s="3">
         <v>50009</v>
       </c>
     </row>
@@ -582,20 +555,21 @@
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="31" customWidth="1"/>
+    <col min="4" max="4" width="21" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
         <v>13</v>
-      </c>
-      <c r="B1" t="s">
-        <v>14</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -603,13 +577,13 @@
         <v>2.25</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated per Zac's recent push to Google-POC branch
</commit_message>
<xml_diff>
--- a/ProvarProject/templates/TestData.xlsx
+++ b/ProvarProject/templates/TestData.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zac.taylor/git/POC-Google/GooglePOC/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27599374-EBC4-3A44-AB06-17B57020C812}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31FF8908-E3E8-5D4A-A9FC-BE36543B5FE5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26320" yWindow="2540" windowWidth="24580" windowHeight="17440" activeTab="1" xr2:uid="{7581156E-45D0-5844-9C4C-1E315867C4A1}"/>
+    <workbookView xWindow="-26320" yWindow="2520" windowWidth="24580" windowHeight="17440" activeTab="2" xr2:uid="{7581156E-45D0-5844-9C4C-1E315867C4A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Fill" sheetId="1" r:id="rId1"/>
     <sheet name="TotalPUF" sheetId="2" r:id="rId2"/>
     <sheet name="SSR" sheetId="3" r:id="rId3"/>
+    <sheet name="FPT" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
   <si>
     <t>GSKU</t>
   </si>
@@ -77,10 +78,25 @@
     <t>Override</t>
   </si>
   <si>
-    <t>Reason</t>
-  </si>
-  <si>
     <t>Units</t>
+  </si>
+  <si>
+    <t>AT20003</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>AT10037</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>PSwift 1.5</t>
+  </si>
+  <si>
+    <t>Notes</t>
   </si>
 </sst>
 </file>
@@ -125,11 +141,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -526,7 +543,7 @@
         <v>11</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -550,40 +567,81 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{816A0B5E-7679-AE41-9C89-C0B5D45A1D99}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="31" customWidth="1"/>
-    <col min="4" max="4" width="21" customWidth="1"/>
+    <col min="2" max="2" width="31" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>12</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2.25</v>
       </c>
       <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B89E2E5-E528-2B46-87B4-96FCDC0E6D22}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" t="s">
         <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>